<commit_message>
data: record climate scenario for IMPACT hunger projections
Primary Climate Inputs now states HadGEM GCM under RCP8.5 with SSP2
socioeconomics, confirmed verbatim from GFPR 2022 Chapter 14
(doi:10.2499/9780896294257_14) - the Dataverse record omits it and the
readme is download-gated. Report artifacts re-rendered.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/submissions/IFPRI.xlsx
+++ b/data/submissions/IFPRI.xlsx
@@ -3507,6 +3507,15 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="K22" s="8" t="inlineStr">
         <is>
@@ -3514,6 +3523,20 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="M37" s="8" t="inlineStr">
         <is>
@@ -3535,6 +3558,11 @@
       <c r="E38" t="inlineStr">
         <is>
           <t>Population at risk of hunger (millions)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>HadGEM GCM under RCP8.5; SSP2 socioeconomics (per 2022 GFPR Ch.14, doi:10.2499/9780896294257_14)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">

</xml_diff>